<commit_message>
Timesheet: 4 job lines per day with daily totals
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01WkobnVQXdGo996siArThhM
</commit_message>
<xml_diff>
--- a/Weekly_Timesheet_Hannah_Plumbing.xlsx
+++ b/Weekly_Timesheet_Hannah_Plumbing.xlsx
@@ -12,8 +12,8 @@
     <sheet name="Example" sheetId="2" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName function="false" hidden="false" localSheetId="1" name="_xlnm.Print_Area" vbProcedure="false">Example!$A$1:$H$33</definedName>
-    <definedName function="false" hidden="false" localSheetId="0" name="_xlnm.Print_Area" vbProcedure="false">Timesheet!$A$1:$H$33</definedName>
+    <definedName function="false" hidden="false" localSheetId="1" name="_xlnm.Print_Area" vbProcedure="false">Example!$A$1:$I$54</definedName>
+    <definedName function="false" hidden="false" localSheetId="0" name="_xlnm.Print_Area" vbProcedure="false">Timesheet!$A$1:$I$54</definedName>
   </definedNames>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -69,7 +69,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="85" uniqueCount="44">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="89" uniqueCount="46">
   <si>
     <t xml:space="preserve">HANNAH PLUMBING &amp; HEATING LTD - WEEKLY TIMESHEET</t>
   </si>
@@ -116,6 +116,9 @@
     <t xml:space="preserve">Hours</t>
   </si>
   <si>
+    <t xml:space="preserve">Day total</t>
+  </si>
+  <si>
     <t xml:space="preserve">Notes (travel, holiday, sick etc.)</t>
   </si>
   <si>
@@ -186,6 +189,9 @@
   </si>
   <si>
     <t xml:space="preserve">Life Church, Paisley - 1st fix</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Boiler service - 12 High St</t>
   </si>
   <si>
     <t xml:space="preserve">Pivot Centre - plant room</t>
@@ -385,7 +391,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="26">
+  <cellXfs count="27">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -430,12 +436,12 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="167" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="167" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="168" fontId="7" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
@@ -450,12 +456,16 @@
       <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="170" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
     <xf numFmtId="164" fontId="6" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="170" fontId="6" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+    <xf numFmtId="170" fontId="6" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="5" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
@@ -742,7 +752,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
-  <dimension ref="A1:H33"/>
+  <dimension ref="A1:I54"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="13"/>
@@ -750,7 +760,8 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="30"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="4" style="0" width="10"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="6" style="0" width="11"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="30"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="10"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="0" width="30"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -769,6 +780,7 @@
       <c r="F2" s="2"/>
       <c r="G2" s="2"/>
       <c r="H2" s="2"/>
+      <c r="I2" s="2"/>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="3" t="s">
@@ -836,10 +848,13 @@
       <c r="H8" s="8" t="s">
         <v>15</v>
       </c>
+      <c r="I8" s="8" t="s">
+        <v>16</v>
+      </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="9" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="B9" s="10"/>
       <c r="C9" s="10"/>
@@ -848,10 +863,11 @@
       <c r="F9" s="10"/>
       <c r="G9" s="10"/>
       <c r="H9" s="10"/>
-    </row>
-    <row r="10" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="I9" s="10"/>
+    </row>
+    <row r="10" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="11" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="B10" s="12" t="str">
         <f aca="false">IF($C$6="","",$C$6+0)</f>
@@ -865,16 +881,15 @@
         <f aca="false">IF(OR(D10="",E10=""),0,MAX(0,MOD(E10-D10,1)*24-N(F10)/60))</f>
         <v>0</v>
       </c>
-      <c r="H10" s="4"/>
-    </row>
-    <row r="11" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A11" s="11" t="s">
-        <v>18</v>
-      </c>
-      <c r="B11" s="12" t="str">
-        <f aca="false">IF($C$6="","",$C$6+1)</f>
-        <v/>
-      </c>
+      <c r="H10" s="16" t="n">
+        <f aca="false">SUM(G10:G13)</f>
+        <v>0</v>
+      </c>
+      <c r="I10" s="4"/>
+    </row>
+    <row r="11" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A11" s="11"/>
+      <c r="B11" s="11"/>
       <c r="C11" s="4"/>
       <c r="D11" s="13"/>
       <c r="E11" s="13"/>
@@ -883,16 +898,12 @@
         <f aca="false">IF(OR(D11="",E11=""),0,MAX(0,MOD(E11-D11,1)*24-N(F11)/60))</f>
         <v>0</v>
       </c>
-      <c r="H11" s="4"/>
-    </row>
-    <row r="12" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A12" s="11" t="s">
-        <v>19</v>
-      </c>
-      <c r="B12" s="12" t="str">
-        <f aca="false">IF($C$6="","",$C$6+2)</f>
-        <v/>
-      </c>
+      <c r="H11" s="16"/>
+      <c r="I11" s="4"/>
+    </row>
+    <row r="12" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A12" s="11"/>
+      <c r="B12" s="11"/>
       <c r="C12" s="4"/>
       <c r="D12" s="13"/>
       <c r="E12" s="13"/>
@@ -901,16 +912,12 @@
         <f aca="false">IF(OR(D12="",E12=""),0,MAX(0,MOD(E12-D12,1)*24-N(F12)/60))</f>
         <v>0</v>
       </c>
-      <c r="H12" s="4"/>
-    </row>
-    <row r="13" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A13" s="11" t="s">
-        <v>20</v>
-      </c>
-      <c r="B13" s="12" t="str">
-        <f aca="false">IF($C$6="","",$C$6+3)</f>
-        <v/>
-      </c>
+      <c r="H12" s="16"/>
+      <c r="I12" s="4"/>
+    </row>
+    <row r="13" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A13" s="11"/>
+      <c r="B13" s="11"/>
       <c r="C13" s="4"/>
       <c r="D13" s="13"/>
       <c r="E13" s="13"/>
@@ -919,14 +926,15 @@
         <f aca="false">IF(OR(D13="",E13=""),0,MAX(0,MOD(E13-D13,1)*24-N(F13)/60))</f>
         <v>0</v>
       </c>
-      <c r="H13" s="4"/>
-    </row>
-    <row r="14" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="H13" s="16"/>
+      <c r="I13" s="4"/>
+    </row>
+    <row r="14" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="11" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="B14" s="12" t="str">
-        <f aca="false">IF($C$6="","",$C$6+4)</f>
+        <f aca="false">IF($C$6="","",$C$6+1)</f>
         <v/>
       </c>
       <c r="C14" s="4"/>
@@ -937,41 +945,60 @@
         <f aca="false">IF(OR(D14="",E14=""),0,MAX(0,MOD(E14-D14,1)*24-N(F14)/60))</f>
         <v>0</v>
       </c>
-      <c r="H14" s="4"/>
-    </row>
-    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="16" t="s">
-        <v>22</v>
-      </c>
-      <c r="B15" s="16"/>
-      <c r="C15" s="16"/>
-      <c r="D15" s="16"/>
-      <c r="E15" s="16"/>
-      <c r="F15" s="16"/>
-      <c r="G15" s="17" t="n">
-        <f aca="false">SUM(G10:G14)</f>
-        <v>0</v>
-      </c>
-      <c r="H15" s="18"/>
-    </row>
-    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="9" t="s">
-        <v>23</v>
-      </c>
-      <c r="B17" s="10"/>
-      <c r="C17" s="10"/>
-      <c r="D17" s="10"/>
-      <c r="E17" s="10"/>
-      <c r="F17" s="10"/>
-      <c r="G17" s="10"/>
-      <c r="H17" s="10"/>
-    </row>
-    <row r="18" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="H14" s="16" t="n">
+        <f aca="false">SUM(G14:G17)</f>
+        <v>0</v>
+      </c>
+      <c r="I14" s="4"/>
+    </row>
+    <row r="15" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A15" s="11"/>
+      <c r="B15" s="11"/>
+      <c r="C15" s="4"/>
+      <c r="D15" s="13"/>
+      <c r="E15" s="13"/>
+      <c r="F15" s="14"/>
+      <c r="G15" s="15" t="n">
+        <f aca="false">IF(OR(D15="",E15=""),0,MAX(0,MOD(E15-D15,1)*24-N(F15)/60))</f>
+        <v>0</v>
+      </c>
+      <c r="H15" s="16"/>
+      <c r="I15" s="4"/>
+    </row>
+    <row r="16" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A16" s="11"/>
+      <c r="B16" s="11"/>
+      <c r="C16" s="4"/>
+      <c r="D16" s="13"/>
+      <c r="E16" s="13"/>
+      <c r="F16" s="14"/>
+      <c r="G16" s="15" t="n">
+        <f aca="false">IF(OR(D16="",E16=""),0,MAX(0,MOD(E16-D16,1)*24-N(F16)/60))</f>
+        <v>0</v>
+      </c>
+      <c r="H16" s="16"/>
+      <c r="I16" s="4"/>
+    </row>
+    <row r="17" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A17" s="11"/>
+      <c r="B17" s="11"/>
+      <c r="C17" s="4"/>
+      <c r="D17" s="13"/>
+      <c r="E17" s="13"/>
+      <c r="F17" s="14"/>
+      <c r="G17" s="15" t="n">
+        <f aca="false">IF(OR(D17="",E17=""),0,MAX(0,MOD(E17-D17,1)*24-N(F17)/60))</f>
+        <v>0</v>
+      </c>
+      <c r="H17" s="16"/>
+      <c r="I17" s="4"/>
+    </row>
+    <row r="18" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="11" t="s">
-        <v>24</v>
+        <v>20</v>
       </c>
       <c r="B18" s="12" t="str">
-        <f aca="false">IF($C$6="","",$C$6+5)</f>
+        <f aca="false">IF($C$6="","",$C$6+2)</f>
         <v/>
       </c>
       <c r="C18" s="4"/>
@@ -982,16 +1009,15 @@
         <f aca="false">IF(OR(D18="",E18=""),0,MAX(0,MOD(E18-D18,1)*24-N(F18)/60))</f>
         <v>0</v>
       </c>
-      <c r="H18" s="4"/>
-    </row>
-    <row r="19" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A19" s="11" t="s">
-        <v>25</v>
-      </c>
-      <c r="B19" s="12" t="str">
-        <f aca="false">IF($C$6="","",$C$6+6)</f>
-        <v/>
-      </c>
+      <c r="H18" s="16" t="n">
+        <f aca="false">SUM(G18:G21)</f>
+        <v>0</v>
+      </c>
+      <c r="I18" s="4"/>
+    </row>
+    <row r="19" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A19" s="11"/>
+      <c r="B19" s="11"/>
       <c r="C19" s="4"/>
       <c r="D19" s="13"/>
       <c r="E19" s="13"/>
@@ -1000,134 +1026,476 @@
         <f aca="false">IF(OR(D19="",E19=""),0,MAX(0,MOD(E19-D19,1)*24-N(F19)/60))</f>
         <v>0</v>
       </c>
-      <c r="H19" s="4"/>
-    </row>
-    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="16" t="s">
+      <c r="H19" s="16"/>
+      <c r="I19" s="4"/>
+    </row>
+    <row r="20" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A20" s="11"/>
+      <c r="B20" s="11"/>
+      <c r="C20" s="4"/>
+      <c r="D20" s="13"/>
+      <c r="E20" s="13"/>
+      <c r="F20" s="14"/>
+      <c r="G20" s="15" t="n">
+        <f aca="false">IF(OR(D20="",E20=""),0,MAX(0,MOD(E20-D20,1)*24-N(F20)/60))</f>
+        <v>0</v>
+      </c>
+      <c r="H20" s="16"/>
+      <c r="I20" s="4"/>
+    </row>
+    <row r="21" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A21" s="11"/>
+      <c r="B21" s="11"/>
+      <c r="C21" s="4"/>
+      <c r="D21" s="13"/>
+      <c r="E21" s="13"/>
+      <c r="F21" s="14"/>
+      <c r="G21" s="15" t="n">
+        <f aca="false">IF(OR(D21="",E21=""),0,MAX(0,MOD(E21-D21,1)*24-N(F21)/60))</f>
+        <v>0</v>
+      </c>
+      <c r="H21" s="16"/>
+      <c r="I21" s="4"/>
+    </row>
+    <row r="22" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A22" s="11" t="s">
+        <v>21</v>
+      </c>
+      <c r="B22" s="12" t="str">
+        <f aca="false">IF($C$6="","",$C$6+3)</f>
+        <v/>
+      </c>
+      <c r="C22" s="4"/>
+      <c r="D22" s="13"/>
+      <c r="E22" s="13"/>
+      <c r="F22" s="14"/>
+      <c r="G22" s="15" t="n">
+        <f aca="false">IF(OR(D22="",E22=""),0,MAX(0,MOD(E22-D22,1)*24-N(F22)/60))</f>
+        <v>0</v>
+      </c>
+      <c r="H22" s="16" t="n">
+        <f aca="false">SUM(G22:G25)</f>
+        <v>0</v>
+      </c>
+      <c r="I22" s="4"/>
+    </row>
+    <row r="23" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A23" s="11"/>
+      <c r="B23" s="11"/>
+      <c r="C23" s="4"/>
+      <c r="D23" s="13"/>
+      <c r="E23" s="13"/>
+      <c r="F23" s="14"/>
+      <c r="G23" s="15" t="n">
+        <f aca="false">IF(OR(D23="",E23=""),0,MAX(0,MOD(E23-D23,1)*24-N(F23)/60))</f>
+        <v>0</v>
+      </c>
+      <c r="H23" s="16"/>
+      <c r="I23" s="4"/>
+    </row>
+    <row r="24" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A24" s="11"/>
+      <c r="B24" s="11"/>
+      <c r="C24" s="4"/>
+      <c r="D24" s="13"/>
+      <c r="E24" s="13"/>
+      <c r="F24" s="14"/>
+      <c r="G24" s="15" t="n">
+        <f aca="false">IF(OR(D24="",E24=""),0,MAX(0,MOD(E24-D24,1)*24-N(F24)/60))</f>
+        <v>0</v>
+      </c>
+      <c r="H24" s="16"/>
+      <c r="I24" s="4"/>
+    </row>
+    <row r="25" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A25" s="11"/>
+      <c r="B25" s="11"/>
+      <c r="C25" s="4"/>
+      <c r="D25" s="13"/>
+      <c r="E25" s="13"/>
+      <c r="F25" s="14"/>
+      <c r="G25" s="15" t="n">
+        <f aca="false">IF(OR(D25="",E25=""),0,MAX(0,MOD(E25-D25,1)*24-N(F25)/60))</f>
+        <v>0</v>
+      </c>
+      <c r="H25" s="16"/>
+      <c r="I25" s="4"/>
+    </row>
+    <row r="26" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A26" s="11" t="s">
+        <v>22</v>
+      </c>
+      <c r="B26" s="12" t="str">
+        <f aca="false">IF($C$6="","",$C$6+4)</f>
+        <v/>
+      </c>
+      <c r="C26" s="4"/>
+      <c r="D26" s="13"/>
+      <c r="E26" s="13"/>
+      <c r="F26" s="14"/>
+      <c r="G26" s="15" t="n">
+        <f aca="false">IF(OR(D26="",E26=""),0,MAX(0,MOD(E26-D26,1)*24-N(F26)/60))</f>
+        <v>0</v>
+      </c>
+      <c r="H26" s="16" t="n">
+        <f aca="false">SUM(G26:G29)</f>
+        <v>0</v>
+      </c>
+      <c r="I26" s="4"/>
+    </row>
+    <row r="27" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A27" s="11"/>
+      <c r="B27" s="11"/>
+      <c r="C27" s="4"/>
+      <c r="D27" s="13"/>
+      <c r="E27" s="13"/>
+      <c r="F27" s="14"/>
+      <c r="G27" s="15" t="n">
+        <f aca="false">IF(OR(D27="",E27=""),0,MAX(0,MOD(E27-D27,1)*24-N(F27)/60))</f>
+        <v>0</v>
+      </c>
+      <c r="H27" s="16"/>
+      <c r="I27" s="4"/>
+    </row>
+    <row r="28" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A28" s="11"/>
+      <c r="B28" s="11"/>
+      <c r="C28" s="4"/>
+      <c r="D28" s="13"/>
+      <c r="E28" s="13"/>
+      <c r="F28" s="14"/>
+      <c r="G28" s="15" t="n">
+        <f aca="false">IF(OR(D28="",E28=""),0,MAX(0,MOD(E28-D28,1)*24-N(F28)/60))</f>
+        <v>0</v>
+      </c>
+      <c r="H28" s="16"/>
+      <c r="I28" s="4"/>
+    </row>
+    <row r="29" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A29" s="11"/>
+      <c r="B29" s="11"/>
+      <c r="C29" s="4"/>
+      <c r="D29" s="13"/>
+      <c r="E29" s="13"/>
+      <c r="F29" s="14"/>
+      <c r="G29" s="15" t="n">
+        <f aca="false">IF(OR(D29="",E29=""),0,MAX(0,MOD(E29-D29,1)*24-N(F29)/60))</f>
+        <v>0</v>
+      </c>
+      <c r="H29" s="16"/>
+      <c r="I29" s="4"/>
+    </row>
+    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A30" s="17" t="s">
+        <v>23</v>
+      </c>
+      <c r="B30" s="17"/>
+      <c r="C30" s="17"/>
+      <c r="D30" s="17"/>
+      <c r="E30" s="17"/>
+      <c r="F30" s="17"/>
+      <c r="G30" s="17"/>
+      <c r="H30" s="18" t="n">
+        <f aca="false">SUM(G10:G29)</f>
+        <v>0</v>
+      </c>
+      <c r="I30" s="19"/>
+    </row>
+    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A32" s="9" t="s">
+        <v>24</v>
+      </c>
+      <c r="B32" s="10"/>
+      <c r="C32" s="10"/>
+      <c r="D32" s="10"/>
+      <c r="E32" s="10"/>
+      <c r="F32" s="10"/>
+      <c r="G32" s="10"/>
+      <c r="H32" s="10"/>
+      <c r="I32" s="10"/>
+    </row>
+    <row r="33" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A33" s="11" t="s">
+        <v>25</v>
+      </c>
+      <c r="B33" s="12" t="str">
+        <f aca="false">IF($C$6="","",$C$6+5)</f>
+        <v/>
+      </c>
+      <c r="C33" s="4"/>
+      <c r="D33" s="13"/>
+      <c r="E33" s="13"/>
+      <c r="F33" s="14"/>
+      <c r="G33" s="15" t="n">
+        <f aca="false">IF(OR(D33="",E33=""),0,MAX(0,MOD(E33-D33,1)*24-N(F33)/60))</f>
+        <v>0</v>
+      </c>
+      <c r="H33" s="16" t="n">
+        <f aca="false">SUM(G33:G36)</f>
+        <v>0</v>
+      </c>
+      <c r="I33" s="4"/>
+    </row>
+    <row r="34" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A34" s="11"/>
+      <c r="B34" s="11"/>
+      <c r="C34" s="4"/>
+      <c r="D34" s="13"/>
+      <c r="E34" s="13"/>
+      <c r="F34" s="14"/>
+      <c r="G34" s="15" t="n">
+        <f aca="false">IF(OR(D34="",E34=""),0,MAX(0,MOD(E34-D34,1)*24-N(F34)/60))</f>
+        <v>0</v>
+      </c>
+      <c r="H34" s="16"/>
+      <c r="I34" s="4"/>
+    </row>
+    <row r="35" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A35" s="11"/>
+      <c r="B35" s="11"/>
+      <c r="C35" s="4"/>
+      <c r="D35" s="13"/>
+      <c r="E35" s="13"/>
+      <c r="F35" s="14"/>
+      <c r="G35" s="15" t="n">
+        <f aca="false">IF(OR(D35="",E35=""),0,MAX(0,MOD(E35-D35,1)*24-N(F35)/60))</f>
+        <v>0</v>
+      </c>
+      <c r="H35" s="16"/>
+      <c r="I35" s="4"/>
+    </row>
+    <row r="36" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A36" s="11"/>
+      <c r="B36" s="11"/>
+      <c r="C36" s="4"/>
+      <c r="D36" s="13"/>
+      <c r="E36" s="13"/>
+      <c r="F36" s="14"/>
+      <c r="G36" s="15" t="n">
+        <f aca="false">IF(OR(D36="",E36=""),0,MAX(0,MOD(E36-D36,1)*24-N(F36)/60))</f>
+        <v>0</v>
+      </c>
+      <c r="H36" s="16"/>
+      <c r="I36" s="4"/>
+    </row>
+    <row r="37" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A37" s="11" t="s">
         <v>26</v>
       </c>
-      <c r="B20" s="16"/>
-      <c r="C20" s="16"/>
-      <c r="D20" s="16"/>
-      <c r="E20" s="16"/>
-      <c r="F20" s="16"/>
-      <c r="G20" s="17" t="n">
-        <f aca="false">SUM(G18:G19)</f>
-        <v>0</v>
-      </c>
-      <c r="H20" s="18"/>
-    </row>
-    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="19" t="s">
+      <c r="B37" s="12" t="str">
+        <f aca="false">IF($C$6="","",$C$6+6)</f>
+        <v/>
+      </c>
+      <c r="C37" s="4"/>
+      <c r="D37" s="13"/>
+      <c r="E37" s="13"/>
+      <c r="F37" s="14"/>
+      <c r="G37" s="15" t="n">
+        <f aca="false">IF(OR(D37="",E37=""),0,MAX(0,MOD(E37-D37,1)*24-N(F37)/60))</f>
+        <v>0</v>
+      </c>
+      <c r="H37" s="16" t="n">
+        <f aca="false">SUM(G37:G40)</f>
+        <v>0</v>
+      </c>
+      <c r="I37" s="4"/>
+    </row>
+    <row r="38" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A38" s="11"/>
+      <c r="B38" s="11"/>
+      <c r="C38" s="4"/>
+      <c r="D38" s="13"/>
+      <c r="E38" s="13"/>
+      <c r="F38" s="14"/>
+      <c r="G38" s="15" t="n">
+        <f aca="false">IF(OR(D38="",E38=""),0,MAX(0,MOD(E38-D38,1)*24-N(F38)/60))</f>
+        <v>0</v>
+      </c>
+      <c r="H38" s="16"/>
+      <c r="I38" s="4"/>
+    </row>
+    <row r="39" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A39" s="11"/>
+      <c r="B39" s="11"/>
+      <c r="C39" s="4"/>
+      <c r="D39" s="13"/>
+      <c r="E39" s="13"/>
+      <c r="F39" s="14"/>
+      <c r="G39" s="15" t="n">
+        <f aca="false">IF(OR(D39="",E39=""),0,MAX(0,MOD(E39-D39,1)*24-N(F39)/60))</f>
+        <v>0</v>
+      </c>
+      <c r="H39" s="16"/>
+      <c r="I39" s="4"/>
+    </row>
+    <row r="40" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A40" s="11"/>
+      <c r="B40" s="11"/>
+      <c r="C40" s="4"/>
+      <c r="D40" s="13"/>
+      <c r="E40" s="13"/>
+      <c r="F40" s="14"/>
+      <c r="G40" s="15" t="n">
+        <f aca="false">IF(OR(D40="",E40=""),0,MAX(0,MOD(E40-D40,1)*24-N(F40)/60))</f>
+        <v>0</v>
+      </c>
+      <c r="H40" s="16"/>
+      <c r="I40" s="4"/>
+    </row>
+    <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A41" s="17" t="s">
         <v>27</v>
       </c>
-    </row>
-    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="20" t="s">
+      <c r="B41" s="17"/>
+      <c r="C41" s="17"/>
+      <c r="D41" s="17"/>
+      <c r="E41" s="17"/>
+      <c r="F41" s="17"/>
+      <c r="G41" s="17"/>
+      <c r="H41" s="18" t="n">
+        <f aca="false">SUM(G33:G40)</f>
+        <v>0</v>
+      </c>
+      <c r="I41" s="19"/>
+    </row>
+    <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A43" s="20" t="s">
         <v>28</v>
       </c>
-      <c r="B23" s="20"/>
-      <c r="C23" s="20"/>
-      <c r="D23" s="20"/>
-      <c r="E23" s="20"/>
-      <c r="F23" s="20"/>
-      <c r="G23" s="21" t="n">
-        <f aca="false">MIN(G15,G4)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A24" s="20" t="s">
+    </row>
+    <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A44" s="21" t="s">
         <v>29</v>
       </c>
-      <c r="B24" s="20"/>
-      <c r="C24" s="20"/>
-      <c r="D24" s="20"/>
-      <c r="E24" s="20"/>
-      <c r="F24" s="20"/>
-      <c r="G24" s="21" t="n">
-        <f aca="false">MAX(0,G15-G4)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A25" s="20" t="s">
+      <c r="B44" s="21"/>
+      <c r="C44" s="21"/>
+      <c r="D44" s="21"/>
+      <c r="E44" s="21"/>
+      <c r="F44" s="21"/>
+      <c r="G44" s="21"/>
+      <c r="H44" s="22" t="n">
+        <f aca="false">MIN(H30,G4)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A45" s="21" t="s">
         <v>30</v>
       </c>
-      <c r="B25" s="20"/>
-      <c r="C25" s="20"/>
-      <c r="D25" s="20"/>
-      <c r="E25" s="20"/>
-      <c r="F25" s="20"/>
-      <c r="G25" s="21" t="n">
-        <f aca="false">G20</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A26" s="9" t="s">
+      <c r="B45" s="21"/>
+      <c r="C45" s="21"/>
+      <c r="D45" s="21"/>
+      <c r="E45" s="21"/>
+      <c r="F45" s="21"/>
+      <c r="G45" s="21"/>
+      <c r="H45" s="22" t="n">
+        <f aca="false">MAX(0,H30-G4)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A46" s="21" t="s">
         <v>31</v>
       </c>
-      <c r="B26" s="9"/>
-      <c r="C26" s="9"/>
-      <c r="D26" s="9"/>
-      <c r="E26" s="9"/>
-      <c r="F26" s="9"/>
-      <c r="G26" s="22" t="n">
-        <f aca="false">G15+G20</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A29" s="23" t="s">
+      <c r="B46" s="21"/>
+      <c r="C46" s="21"/>
+      <c r="D46" s="21"/>
+      <c r="E46" s="21"/>
+      <c r="F46" s="21"/>
+      <c r="G46" s="21"/>
+      <c r="H46" s="22" t="n">
+        <f aca="false">H41</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A47" s="9" t="s">
         <v>32</v>
       </c>
-      <c r="B29" s="24"/>
-      <c r="C29" s="24"/>
-      <c r="D29" s="24"/>
-      <c r="E29" s="23" t="s">
+      <c r="B47" s="9"/>
+      <c r="C47" s="9"/>
+      <c r="D47" s="9"/>
+      <c r="E47" s="9"/>
+      <c r="F47" s="9"/>
+      <c r="G47" s="9"/>
+      <c r="H47" s="23" t="n">
+        <f aca="false">H30+H41</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A50" s="24" t="s">
+        <v>33</v>
+      </c>
+      <c r="B50" s="25"/>
+      <c r="C50" s="25"/>
+      <c r="D50" s="25"/>
+      <c r="E50" s="24" t="s">
         <v>9</v>
       </c>
-      <c r="F29" s="24"/>
-      <c r="G29" s="24"/>
-    </row>
-    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A31" s="23" t="s">
-        <v>33</v>
-      </c>
-      <c r="B31" s="24"/>
-      <c r="C31" s="24"/>
-      <c r="D31" s="24"/>
-      <c r="E31" s="23" t="s">
+      <c r="F50" s="25"/>
+      <c r="G50" s="25"/>
+      <c r="H50" s="25"/>
+    </row>
+    <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A52" s="24" t="s">
+        <v>34</v>
+      </c>
+      <c r="B52" s="25"/>
+      <c r="C52" s="25"/>
+      <c r="D52" s="25"/>
+      <c r="E52" s="24" t="s">
         <v>9</v>
       </c>
-      <c r="F31" s="24"/>
-      <c r="G31" s="24"/>
-    </row>
-    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A33" s="25" t="s">
-        <v>34</v>
+      <c r="F52" s="25"/>
+      <c r="G52" s="25"/>
+      <c r="H52" s="25"/>
+    </row>
+    <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A54" s="26" t="s">
+        <v>35</v>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="13">
-    <mergeCell ref="A2:H2"/>
+  <mergeCells count="34">
+    <mergeCell ref="A2:I2"/>
     <mergeCell ref="A4:B4"/>
     <mergeCell ref="E4:F4"/>
     <mergeCell ref="A5:B5"/>
     <mergeCell ref="E5:F5"/>
     <mergeCell ref="A6:B6"/>
     <mergeCell ref="E6:F6"/>
-    <mergeCell ref="A15:F15"/>
-    <mergeCell ref="A20:F20"/>
-    <mergeCell ref="A23:F23"/>
-    <mergeCell ref="A24:F24"/>
-    <mergeCell ref="A25:F25"/>
-    <mergeCell ref="A26:F26"/>
+    <mergeCell ref="A10:A13"/>
+    <mergeCell ref="B10:B13"/>
+    <mergeCell ref="H10:H13"/>
+    <mergeCell ref="A14:A17"/>
+    <mergeCell ref="B14:B17"/>
+    <mergeCell ref="H14:H17"/>
+    <mergeCell ref="A18:A21"/>
+    <mergeCell ref="B18:B21"/>
+    <mergeCell ref="H18:H21"/>
+    <mergeCell ref="A22:A25"/>
+    <mergeCell ref="B22:B25"/>
+    <mergeCell ref="H22:H25"/>
+    <mergeCell ref="A26:A29"/>
+    <mergeCell ref="B26:B29"/>
+    <mergeCell ref="H26:H29"/>
+    <mergeCell ref="A30:G30"/>
+    <mergeCell ref="A33:A36"/>
+    <mergeCell ref="B33:B36"/>
+    <mergeCell ref="H33:H36"/>
+    <mergeCell ref="A37:A40"/>
+    <mergeCell ref="B37:B40"/>
+    <mergeCell ref="H37:H40"/>
+    <mergeCell ref="A41:G41"/>
+    <mergeCell ref="A44:G44"/>
+    <mergeCell ref="A45:G45"/>
+    <mergeCell ref="A46:G46"/>
+    <mergeCell ref="A47:G47"/>
   </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="landscape" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter differentFirst="false" differentOddEven="false">
     <oddHeader/>
     <oddFooter/>
@@ -1141,7 +1509,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
-  <dimension ref="A1:H33"/>
+  <dimension ref="A1:I54"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="13"/>
@@ -1149,7 +1517,8 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="30"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="4" style="0" width="10"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="6" style="0" width="11"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="30"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="10"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="0" width="30"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1168,6 +1537,7 @@
       <c r="F2" s="2"/>
       <c r="G2" s="2"/>
       <c r="H2" s="2"/>
+      <c r="I2" s="2"/>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="3" t="s">
@@ -1175,7 +1545,7 @@
       </c>
       <c r="B4" s="3"/>
       <c r="C4" s="4" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="E4" s="3" t="s">
         <v>3</v>
@@ -1191,14 +1561,14 @@
       </c>
       <c r="B5" s="3"/>
       <c r="C5" s="4" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="E5" s="3" t="s">
         <v>5</v>
       </c>
       <c r="F5" s="3"/>
       <c r="G5" s="4" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1243,10 +1613,13 @@
       <c r="H8" s="8" t="s">
         <v>15</v>
       </c>
+      <c r="I8" s="8" t="s">
+        <v>16</v>
+      </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="9" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="B9" s="10"/>
       <c r="C9" s="10"/>
@@ -1255,17 +1628,18 @@
       <c r="F9" s="10"/>
       <c r="G9" s="10"/>
       <c r="H9" s="10"/>
-    </row>
-    <row r="10" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="I9" s="10"/>
+    </row>
+    <row r="10" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="11" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="B10" s="12" t="n">
         <f aca="false">IF($C$6="","",$C$6+0)</f>
         <v>46300</v>
       </c>
       <c r="C10" s="4" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="D10" s="13" t="n">
         <v>0.333333333333333</v>
@@ -1280,171 +1654,177 @@
         <f aca="false">IF(OR(D10="",E10=""),0,MAX(0,MOD(E10-D10,1)*24-N(F10)/60))</f>
         <v>8</v>
       </c>
-      <c r="H10" s="4"/>
-    </row>
-    <row r="11" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A11" s="11" t="s">
-        <v>18</v>
-      </c>
-      <c r="B11" s="12" t="n">
+      <c r="H10" s="16" t="n">
+        <f aca="false">SUM(G10:G13)</f>
+        <v>8</v>
+      </c>
+      <c r="I10" s="4"/>
+    </row>
+    <row r="11" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A11" s="11"/>
+      <c r="B11" s="11"/>
+      <c r="C11" s="4"/>
+      <c r="D11" s="13"/>
+      <c r="E11" s="13"/>
+      <c r="F11" s="14"/>
+      <c r="G11" s="15" t="n">
+        <f aca="false">IF(OR(D11="",E11=""),0,MAX(0,MOD(E11-D11,1)*24-N(F11)/60))</f>
+        <v>0</v>
+      </c>
+      <c r="H11" s="16"/>
+      <c r="I11" s="4"/>
+    </row>
+    <row r="12" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A12" s="11"/>
+      <c r="B12" s="11"/>
+      <c r="C12" s="4"/>
+      <c r="D12" s="13"/>
+      <c r="E12" s="13"/>
+      <c r="F12" s="14"/>
+      <c r="G12" s="15" t="n">
+        <f aca="false">IF(OR(D12="",E12=""),0,MAX(0,MOD(E12-D12,1)*24-N(F12)/60))</f>
+        <v>0</v>
+      </c>
+      <c r="H12" s="16"/>
+      <c r="I12" s="4"/>
+    </row>
+    <row r="13" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A13" s="11"/>
+      <c r="B13" s="11"/>
+      <c r="C13" s="4"/>
+      <c r="D13" s="13"/>
+      <c r="E13" s="13"/>
+      <c r="F13" s="14"/>
+      <c r="G13" s="15" t="n">
+        <f aca="false">IF(OR(D13="",E13=""),0,MAX(0,MOD(E13-D13,1)*24-N(F13)/60))</f>
+        <v>0</v>
+      </c>
+      <c r="H13" s="16"/>
+      <c r="I13" s="4"/>
+    </row>
+    <row r="14" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A14" s="11" t="s">
+        <v>19</v>
+      </c>
+      <c r="B14" s="12" t="n">
         <f aca="false">IF($C$6="","",$C$6+1)</f>
         <v>46301</v>
       </c>
-      <c r="C11" s="4" t="s">
-        <v>38</v>
-      </c>
-      <c r="D11" s="13" t="n">
+      <c r="C14" s="4" t="s">
+        <v>39</v>
+      </c>
+      <c r="D14" s="13" t="n">
         <v>0.333333333333333</v>
       </c>
-      <c r="E11" s="13" t="n">
+      <c r="E14" s="13" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="F14" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="G14" s="15" t="n">
+        <f aca="false">IF(OR(D14="",E14=""),0,MAX(0,MOD(E14-D14,1)*24-N(F14)/60))</f>
+        <v>4</v>
+      </c>
+      <c r="H14" s="16" t="n">
+        <f aca="false">SUM(G14:G17)</f>
+        <v>7.75</v>
+      </c>
+      <c r="I14" s="4"/>
+    </row>
+    <row r="15" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A15" s="11"/>
+      <c r="B15" s="11"/>
+      <c r="C15" s="4" t="s">
+        <v>40</v>
+      </c>
+      <c r="D15" s="13" t="n">
+        <v>0.520833333333333</v>
+      </c>
+      <c r="E15" s="13" t="n">
+        <v>0.583333333333333</v>
+      </c>
+      <c r="F15" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="G15" s="15" t="n">
+        <f aca="false">IF(OR(D15="",E15=""),0,MAX(0,MOD(E15-D15,1)*24-N(F15)/60))</f>
+        <v>1.5</v>
+      </c>
+      <c r="H15" s="16"/>
+      <c r="I15" s="4"/>
+    </row>
+    <row r="16" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A16" s="11"/>
+      <c r="B16" s="11"/>
+      <c r="C16" s="4" t="s">
+        <v>39</v>
+      </c>
+      <c r="D16" s="13" t="n">
+        <v>0.59375</v>
+      </c>
+      <c r="E16" s="13" t="n">
         <v>0.6875</v>
       </c>
-      <c r="F11" s="14" t="n">
-        <v>30</v>
-      </c>
-      <c r="G11" s="15" t="n">
-        <f aca="false">IF(OR(D11="",E11=""),0,MAX(0,MOD(E11-D11,1)*24-N(F11)/60))</f>
-        <v>8</v>
-      </c>
-      <c r="H11" s="4"/>
-    </row>
-    <row r="12" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A12" s="11" t="s">
-        <v>19</v>
-      </c>
-      <c r="B12" s="12" t="n">
+      <c r="F16" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="G16" s="15" t="n">
+        <f aca="false">IF(OR(D16="",E16=""),0,MAX(0,MOD(E16-D16,1)*24-N(F16)/60))</f>
+        <v>2.25</v>
+      </c>
+      <c r="H16" s="16"/>
+      <c r="I16" s="4"/>
+    </row>
+    <row r="17" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A17" s="11"/>
+      <c r="B17" s="11"/>
+      <c r="C17" s="4"/>
+      <c r="D17" s="13"/>
+      <c r="E17" s="13"/>
+      <c r="F17" s="14"/>
+      <c r="G17" s="15" t="n">
+        <f aca="false">IF(OR(D17="",E17=""),0,MAX(0,MOD(E17-D17,1)*24-N(F17)/60))</f>
+        <v>0</v>
+      </c>
+      <c r="H17" s="16"/>
+      <c r="I17" s="4"/>
+    </row>
+    <row r="18" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A18" s="11" t="s">
+        <v>20</v>
+      </c>
+      <c r="B18" s="12" t="n">
         <f aca="false">IF($C$6="","",$C$6+2)</f>
         <v>46302</v>
       </c>
-      <c r="C12" s="4" t="s">
-        <v>39</v>
-      </c>
-      <c r="D12" s="13" t="n">
+      <c r="C18" s="4" t="s">
+        <v>41</v>
+      </c>
+      <c r="D18" s="13" t="n">
         <v>0.3125</v>
       </c>
-      <c r="E12" s="13" t="n">
+      <c r="E18" s="13" t="n">
         <v>0.729166666666667</v>
       </c>
-      <c r="F12" s="14" t="n">
+      <c r="F18" s="14" t="n">
         <v>30</v>
-      </c>
-      <c r="G12" s="15" t="n">
-        <f aca="false">IF(OR(D12="",E12=""),0,MAX(0,MOD(E12-D12,1)*24-N(F12)/60))</f>
-        <v>9.5</v>
-      </c>
-      <c r="H12" s="4" t="s">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="13" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A13" s="11" t="s">
-        <v>20</v>
-      </c>
-      <c r="B13" s="12" t="n">
-        <f aca="false">IF($C$6="","",$C$6+3)</f>
-        <v>46303</v>
-      </c>
-      <c r="C13" s="4" t="s">
-        <v>39</v>
-      </c>
-      <c r="D13" s="13" t="n">
-        <v>0.333333333333333</v>
-      </c>
-      <c r="E13" s="13" t="n">
-        <v>0.6875</v>
-      </c>
-      <c r="F13" s="14" t="n">
-        <v>30</v>
-      </c>
-      <c r="G13" s="15" t="n">
-        <f aca="false">IF(OR(D13="",E13=""),0,MAX(0,MOD(E13-D13,1)*24-N(F13)/60))</f>
-        <v>8</v>
-      </c>
-      <c r="H13" s="4"/>
-    </row>
-    <row r="14" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A14" s="11" t="s">
-        <v>21</v>
-      </c>
-      <c r="B14" s="12" t="n">
-        <f aca="false">IF($C$6="","",$C$6+4)</f>
-        <v>46304</v>
-      </c>
-      <c r="C14" s="4"/>
-      <c r="D14" s="13"/>
-      <c r="E14" s="13"/>
-      <c r="F14" s="14"/>
-      <c r="G14" s="15" t="n">
-        <f aca="false">IF(OR(D14="",E14=""),0,MAX(0,MOD(E14-D14,1)*24-N(F14)/60))</f>
-        <v>0</v>
-      </c>
-      <c r="H14" s="4" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="16" t="s">
-        <v>22</v>
-      </c>
-      <c r="B15" s="16"/>
-      <c r="C15" s="16"/>
-      <c r="D15" s="16"/>
-      <c r="E15" s="16"/>
-      <c r="F15" s="16"/>
-      <c r="G15" s="17" t="n">
-        <f aca="false">SUM(G10:G14)</f>
-        <v>33.5</v>
-      </c>
-      <c r="H15" s="18"/>
-    </row>
-    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="9" t="s">
-        <v>23</v>
-      </c>
-      <c r="B17" s="10"/>
-      <c r="C17" s="10"/>
-      <c r="D17" s="10"/>
-      <c r="E17" s="10"/>
-      <c r="F17" s="10"/>
-      <c r="G17" s="10"/>
-      <c r="H17" s="10"/>
-    </row>
-    <row r="18" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A18" s="11" t="s">
-        <v>24</v>
-      </c>
-      <c r="B18" s="12" t="n">
-        <f aca="false">IF($C$6="","",$C$6+5)</f>
-        <v>46305</v>
-      </c>
-      <c r="C18" s="4" t="s">
-        <v>42</v>
-      </c>
-      <c r="D18" s="13" t="n">
-        <v>0.375</v>
-      </c>
-      <c r="E18" s="13" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="F18" s="14" t="n">
-        <v>0</v>
       </c>
       <c r="G18" s="15" t="n">
         <f aca="false">IF(OR(D18="",E18=""),0,MAX(0,MOD(E18-D18,1)*24-N(F18)/60))</f>
-        <v>3</v>
-      </c>
-      <c r="H18" s="4" t="s">
-        <v>43</v>
-      </c>
-    </row>
-    <row r="19" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A19" s="11" t="s">
-        <v>25</v>
-      </c>
-      <c r="B19" s="12" t="n">
-        <f aca="false">IF($C$6="","",$C$6+6)</f>
-        <v>46306</v>
-      </c>
+        <v>9.5</v>
+      </c>
+      <c r="H18" s="16" t="n">
+        <f aca="false">SUM(G18:G21)</f>
+        <v>9.5</v>
+      </c>
+      <c r="I18" s="4" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="19" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A19" s="11"/>
+      <c r="B19" s="11"/>
       <c r="C19" s="4"/>
       <c r="D19" s="13"/>
       <c r="E19" s="13"/>
@@ -1453,134 +1833,496 @@
         <f aca="false">IF(OR(D19="",E19=""),0,MAX(0,MOD(E19-D19,1)*24-N(F19)/60))</f>
         <v>0</v>
       </c>
-      <c r="H19" s="4"/>
-    </row>
-    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="16" t="s">
+      <c r="H19" s="16"/>
+      <c r="I19" s="4"/>
+    </row>
+    <row r="20" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A20" s="11"/>
+      <c r="B20" s="11"/>
+      <c r="C20" s="4"/>
+      <c r="D20" s="13"/>
+      <c r="E20" s="13"/>
+      <c r="F20" s="14"/>
+      <c r="G20" s="15" t="n">
+        <f aca="false">IF(OR(D20="",E20=""),0,MAX(0,MOD(E20-D20,1)*24-N(F20)/60))</f>
+        <v>0</v>
+      </c>
+      <c r="H20" s="16"/>
+      <c r="I20" s="4"/>
+    </row>
+    <row r="21" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A21" s="11"/>
+      <c r="B21" s="11"/>
+      <c r="C21" s="4"/>
+      <c r="D21" s="13"/>
+      <c r="E21" s="13"/>
+      <c r="F21" s="14"/>
+      <c r="G21" s="15" t="n">
+        <f aca="false">IF(OR(D21="",E21=""),0,MAX(0,MOD(E21-D21,1)*24-N(F21)/60))</f>
+        <v>0</v>
+      </c>
+      <c r="H21" s="16"/>
+      <c r="I21" s="4"/>
+    </row>
+    <row r="22" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A22" s="11" t="s">
+        <v>21</v>
+      </c>
+      <c r="B22" s="12" t="n">
+        <f aca="false">IF($C$6="","",$C$6+3)</f>
+        <v>46303</v>
+      </c>
+      <c r="C22" s="4" t="s">
+        <v>41</v>
+      </c>
+      <c r="D22" s="13" t="n">
+        <v>0.333333333333333</v>
+      </c>
+      <c r="E22" s="13" t="n">
+        <v>0.6875</v>
+      </c>
+      <c r="F22" s="14" t="n">
+        <v>30</v>
+      </c>
+      <c r="G22" s="15" t="n">
+        <f aca="false">IF(OR(D22="",E22=""),0,MAX(0,MOD(E22-D22,1)*24-N(F22)/60))</f>
+        <v>8</v>
+      </c>
+      <c r="H22" s="16" t="n">
+        <f aca="false">SUM(G22:G25)</f>
+        <v>8</v>
+      </c>
+      <c r="I22" s="4"/>
+    </row>
+    <row r="23" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A23" s="11"/>
+      <c r="B23" s="11"/>
+      <c r="C23" s="4"/>
+      <c r="D23" s="13"/>
+      <c r="E23" s="13"/>
+      <c r="F23" s="14"/>
+      <c r="G23" s="15" t="n">
+        <f aca="false">IF(OR(D23="",E23=""),0,MAX(0,MOD(E23-D23,1)*24-N(F23)/60))</f>
+        <v>0</v>
+      </c>
+      <c r="H23" s="16"/>
+      <c r="I23" s="4"/>
+    </row>
+    <row r="24" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A24" s="11"/>
+      <c r="B24" s="11"/>
+      <c r="C24" s="4"/>
+      <c r="D24" s="13"/>
+      <c r="E24" s="13"/>
+      <c r="F24" s="14"/>
+      <c r="G24" s="15" t="n">
+        <f aca="false">IF(OR(D24="",E24=""),0,MAX(0,MOD(E24-D24,1)*24-N(F24)/60))</f>
+        <v>0</v>
+      </c>
+      <c r="H24" s="16"/>
+      <c r="I24" s="4"/>
+    </row>
+    <row r="25" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A25" s="11"/>
+      <c r="B25" s="11"/>
+      <c r="C25" s="4"/>
+      <c r="D25" s="13"/>
+      <c r="E25" s="13"/>
+      <c r="F25" s="14"/>
+      <c r="G25" s="15" t="n">
+        <f aca="false">IF(OR(D25="",E25=""),0,MAX(0,MOD(E25-D25,1)*24-N(F25)/60))</f>
+        <v>0</v>
+      </c>
+      <c r="H25" s="16"/>
+      <c r="I25" s="4"/>
+    </row>
+    <row r="26" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A26" s="11" t="s">
+        <v>22</v>
+      </c>
+      <c r="B26" s="12" t="n">
+        <f aca="false">IF($C$6="","",$C$6+4)</f>
+        <v>46304</v>
+      </c>
+      <c r="C26" s="4"/>
+      <c r="D26" s="13"/>
+      <c r="E26" s="13"/>
+      <c r="F26" s="14"/>
+      <c r="G26" s="15" t="n">
+        <f aca="false">IF(OR(D26="",E26=""),0,MAX(0,MOD(E26-D26,1)*24-N(F26)/60))</f>
+        <v>0</v>
+      </c>
+      <c r="H26" s="16" t="n">
+        <f aca="false">SUM(G26:G29)</f>
+        <v>0</v>
+      </c>
+      <c r="I26" s="4" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="27" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A27" s="11"/>
+      <c r="B27" s="11"/>
+      <c r="C27" s="4"/>
+      <c r="D27" s="13"/>
+      <c r="E27" s="13"/>
+      <c r="F27" s="14"/>
+      <c r="G27" s="15" t="n">
+        <f aca="false">IF(OR(D27="",E27=""),0,MAX(0,MOD(E27-D27,1)*24-N(F27)/60))</f>
+        <v>0</v>
+      </c>
+      <c r="H27" s="16"/>
+      <c r="I27" s="4"/>
+    </row>
+    <row r="28" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A28" s="11"/>
+      <c r="B28" s="11"/>
+      <c r="C28" s="4"/>
+      <c r="D28" s="13"/>
+      <c r="E28" s="13"/>
+      <c r="F28" s="14"/>
+      <c r="G28" s="15" t="n">
+        <f aca="false">IF(OR(D28="",E28=""),0,MAX(0,MOD(E28-D28,1)*24-N(F28)/60))</f>
+        <v>0</v>
+      </c>
+      <c r="H28" s="16"/>
+      <c r="I28" s="4"/>
+    </row>
+    <row r="29" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A29" s="11"/>
+      <c r="B29" s="11"/>
+      <c r="C29" s="4"/>
+      <c r="D29" s="13"/>
+      <c r="E29" s="13"/>
+      <c r="F29" s="14"/>
+      <c r="G29" s="15" t="n">
+        <f aca="false">IF(OR(D29="",E29=""),0,MAX(0,MOD(E29-D29,1)*24-N(F29)/60))</f>
+        <v>0</v>
+      </c>
+      <c r="H29" s="16"/>
+      <c r="I29" s="4"/>
+    </row>
+    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A30" s="17" t="s">
+        <v>23</v>
+      </c>
+      <c r="B30" s="17"/>
+      <c r="C30" s="17"/>
+      <c r="D30" s="17"/>
+      <c r="E30" s="17"/>
+      <c r="F30" s="17"/>
+      <c r="G30" s="17"/>
+      <c r="H30" s="18" t="n">
+        <f aca="false">SUM(G10:G29)</f>
+        <v>33.25</v>
+      </c>
+      <c r="I30" s="19"/>
+    </row>
+    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A32" s="9" t="s">
+        <v>24</v>
+      </c>
+      <c r="B32" s="10"/>
+      <c r="C32" s="10"/>
+      <c r="D32" s="10"/>
+      <c r="E32" s="10"/>
+      <c r="F32" s="10"/>
+      <c r="G32" s="10"/>
+      <c r="H32" s="10"/>
+      <c r="I32" s="10"/>
+    </row>
+    <row r="33" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A33" s="11" t="s">
+        <v>25</v>
+      </c>
+      <c r="B33" s="12" t="n">
+        <f aca="false">IF($C$6="","",$C$6+5)</f>
+        <v>46305</v>
+      </c>
+      <c r="C33" s="4" t="s">
+        <v>44</v>
+      </c>
+      <c r="D33" s="13" t="n">
+        <v>0.375</v>
+      </c>
+      <c r="E33" s="13" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="F33" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="G33" s="15" t="n">
+        <f aca="false">IF(OR(D33="",E33=""),0,MAX(0,MOD(E33-D33,1)*24-N(F33)/60))</f>
+        <v>3</v>
+      </c>
+      <c r="H33" s="16" t="n">
+        <f aca="false">SUM(G33:G36)</f>
+        <v>3</v>
+      </c>
+      <c r="I33" s="4" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="34" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A34" s="11"/>
+      <c r="B34" s="11"/>
+      <c r="C34" s="4"/>
+      <c r="D34" s="13"/>
+      <c r="E34" s="13"/>
+      <c r="F34" s="14"/>
+      <c r="G34" s="15" t="n">
+        <f aca="false">IF(OR(D34="",E34=""),0,MAX(0,MOD(E34-D34,1)*24-N(F34)/60))</f>
+        <v>0</v>
+      </c>
+      <c r="H34" s="16"/>
+      <c r="I34" s="4"/>
+    </row>
+    <row r="35" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A35" s="11"/>
+      <c r="B35" s="11"/>
+      <c r="C35" s="4"/>
+      <c r="D35" s="13"/>
+      <c r="E35" s="13"/>
+      <c r="F35" s="14"/>
+      <c r="G35" s="15" t="n">
+        <f aca="false">IF(OR(D35="",E35=""),0,MAX(0,MOD(E35-D35,1)*24-N(F35)/60))</f>
+        <v>0</v>
+      </c>
+      <c r="H35" s="16"/>
+      <c r="I35" s="4"/>
+    </row>
+    <row r="36" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A36" s="11"/>
+      <c r="B36" s="11"/>
+      <c r="C36" s="4"/>
+      <c r="D36" s="13"/>
+      <c r="E36" s="13"/>
+      <c r="F36" s="14"/>
+      <c r="G36" s="15" t="n">
+        <f aca="false">IF(OR(D36="",E36=""),0,MAX(0,MOD(E36-D36,1)*24-N(F36)/60))</f>
+        <v>0</v>
+      </c>
+      <c r="H36" s="16"/>
+      <c r="I36" s="4"/>
+    </row>
+    <row r="37" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A37" s="11" t="s">
         <v>26</v>
       </c>
-      <c r="B20" s="16"/>
-      <c r="C20" s="16"/>
-      <c r="D20" s="16"/>
-      <c r="E20" s="16"/>
-      <c r="F20" s="16"/>
-      <c r="G20" s="17" t="n">
-        <f aca="false">SUM(G18:G19)</f>
+      <c r="B37" s="12" t="n">
+        <f aca="false">IF($C$6="","",$C$6+6)</f>
+        <v>46306</v>
+      </c>
+      <c r="C37" s="4"/>
+      <c r="D37" s="13"/>
+      <c r="E37" s="13"/>
+      <c r="F37" s="14"/>
+      <c r="G37" s="15" t="n">
+        <f aca="false">IF(OR(D37="",E37=""),0,MAX(0,MOD(E37-D37,1)*24-N(F37)/60))</f>
+        <v>0</v>
+      </c>
+      <c r="H37" s="16" t="n">
+        <f aca="false">SUM(G37:G40)</f>
+        <v>0</v>
+      </c>
+      <c r="I37" s="4"/>
+    </row>
+    <row r="38" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A38" s="11"/>
+      <c r="B38" s="11"/>
+      <c r="C38" s="4"/>
+      <c r="D38" s="13"/>
+      <c r="E38" s="13"/>
+      <c r="F38" s="14"/>
+      <c r="G38" s="15" t="n">
+        <f aca="false">IF(OR(D38="",E38=""),0,MAX(0,MOD(E38-D38,1)*24-N(F38)/60))</f>
+        <v>0</v>
+      </c>
+      <c r="H38" s="16"/>
+      <c r="I38" s="4"/>
+    </row>
+    <row r="39" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A39" s="11"/>
+      <c r="B39" s="11"/>
+      <c r="C39" s="4"/>
+      <c r="D39" s="13"/>
+      <c r="E39" s="13"/>
+      <c r="F39" s="14"/>
+      <c r="G39" s="15" t="n">
+        <f aca="false">IF(OR(D39="",E39=""),0,MAX(0,MOD(E39-D39,1)*24-N(F39)/60))</f>
+        <v>0</v>
+      </c>
+      <c r="H39" s="16"/>
+      <c r="I39" s="4"/>
+    </row>
+    <row r="40" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A40" s="11"/>
+      <c r="B40" s="11"/>
+      <c r="C40" s="4"/>
+      <c r="D40" s="13"/>
+      <c r="E40" s="13"/>
+      <c r="F40" s="14"/>
+      <c r="G40" s="15" t="n">
+        <f aca="false">IF(OR(D40="",E40=""),0,MAX(0,MOD(E40-D40,1)*24-N(F40)/60))</f>
+        <v>0</v>
+      </c>
+      <c r="H40" s="16"/>
+      <c r="I40" s="4"/>
+    </row>
+    <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A41" s="17" t="s">
+        <v>27</v>
+      </c>
+      <c r="B41" s="17"/>
+      <c r="C41" s="17"/>
+      <c r="D41" s="17"/>
+      <c r="E41" s="17"/>
+      <c r="F41" s="17"/>
+      <c r="G41" s="17"/>
+      <c r="H41" s="18" t="n">
+        <f aca="false">SUM(G33:G40)</f>
         <v>3</v>
       </c>
-      <c r="H20" s="18"/>
-    </row>
-    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="19" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="20" t="s">
+      <c r="I41" s="19"/>
+    </row>
+    <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A43" s="20" t="s">
         <v>28</v>
       </c>
-      <c r="B23" s="20"/>
-      <c r="C23" s="20"/>
-      <c r="D23" s="20"/>
-      <c r="E23" s="20"/>
-      <c r="F23" s="20"/>
-      <c r="G23" s="21" t="n">
-        <f aca="false">MIN(G15,G4)</f>
-        <v>33.5</v>
-      </c>
-    </row>
-    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A24" s="20" t="s">
+    </row>
+    <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A44" s="21" t="s">
         <v>29</v>
       </c>
-      <c r="B24" s="20"/>
-      <c r="C24" s="20"/>
-      <c r="D24" s="20"/>
-      <c r="E24" s="20"/>
-      <c r="F24" s="20"/>
-      <c r="G24" s="21" t="n">
-        <f aca="false">MAX(0,G15-G4)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A25" s="20" t="s">
+      <c r="B44" s="21"/>
+      <c r="C44" s="21"/>
+      <c r="D44" s="21"/>
+      <c r="E44" s="21"/>
+      <c r="F44" s="21"/>
+      <c r="G44" s="21"/>
+      <c r="H44" s="22" t="n">
+        <f aca="false">MIN(H30,G4)</f>
+        <v>33.25</v>
+      </c>
+    </row>
+    <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A45" s="21" t="s">
         <v>30</v>
       </c>
-      <c r="B25" s="20"/>
-      <c r="C25" s="20"/>
-      <c r="D25" s="20"/>
-      <c r="E25" s="20"/>
-      <c r="F25" s="20"/>
-      <c r="G25" s="21" t="n">
-        <f aca="false">G20</f>
+      <c r="B45" s="21"/>
+      <c r="C45" s="21"/>
+      <c r="D45" s="21"/>
+      <c r="E45" s="21"/>
+      <c r="F45" s="21"/>
+      <c r="G45" s="21"/>
+      <c r="H45" s="22" t="n">
+        <f aca="false">MAX(0,H30-G4)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A46" s="21" t="s">
+        <v>31</v>
+      </c>
+      <c r="B46" s="21"/>
+      <c r="C46" s="21"/>
+      <c r="D46" s="21"/>
+      <c r="E46" s="21"/>
+      <c r="F46" s="21"/>
+      <c r="G46" s="21"/>
+      <c r="H46" s="22" t="n">
+        <f aca="false">H41</f>
         <v>3</v>
       </c>
     </row>
-    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A26" s="9" t="s">
-        <v>31</v>
-      </c>
-      <c r="B26" s="9"/>
-      <c r="C26" s="9"/>
-      <c r="D26" s="9"/>
-      <c r="E26" s="9"/>
-      <c r="F26" s="9"/>
-      <c r="G26" s="22" t="n">
-        <f aca="false">G15+G20</f>
-        <v>36.5</v>
-      </c>
-    </row>
-    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A29" s="23" t="s">
+    <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A47" s="9" t="s">
         <v>32</v>
       </c>
-      <c r="B29" s="24"/>
-      <c r="C29" s="24"/>
-      <c r="D29" s="24"/>
-      <c r="E29" s="23" t="s">
+      <c r="B47" s="9"/>
+      <c r="C47" s="9"/>
+      <c r="D47" s="9"/>
+      <c r="E47" s="9"/>
+      <c r="F47" s="9"/>
+      <c r="G47" s="9"/>
+      <c r="H47" s="23" t="n">
+        <f aca="false">H30+H41</f>
+        <v>36.25</v>
+      </c>
+    </row>
+    <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A50" s="24" t="s">
+        <v>33</v>
+      </c>
+      <c r="B50" s="25"/>
+      <c r="C50" s="25"/>
+      <c r="D50" s="25"/>
+      <c r="E50" s="24" t="s">
         <v>9</v>
       </c>
-      <c r="F29" s="24"/>
-      <c r="G29" s="24"/>
-    </row>
-    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A31" s="23" t="s">
-        <v>33</v>
-      </c>
-      <c r="B31" s="24"/>
-      <c r="C31" s="24"/>
-      <c r="D31" s="24"/>
-      <c r="E31" s="23" t="s">
+      <c r="F50" s="25"/>
+      <c r="G50" s="25"/>
+      <c r="H50" s="25"/>
+    </row>
+    <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A52" s="24" t="s">
+        <v>34</v>
+      </c>
+      <c r="B52" s="25"/>
+      <c r="C52" s="25"/>
+      <c r="D52" s="25"/>
+      <c r="E52" s="24" t="s">
         <v>9</v>
       </c>
-      <c r="F31" s="24"/>
-      <c r="G31" s="24"/>
-    </row>
-    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A33" s="25" t="s">
-        <v>34</v>
+      <c r="F52" s="25"/>
+      <c r="G52" s="25"/>
+      <c r="H52" s="25"/>
+    </row>
+    <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A54" s="26" t="s">
+        <v>35</v>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="13">
-    <mergeCell ref="A2:H2"/>
+  <mergeCells count="34">
+    <mergeCell ref="A2:I2"/>
     <mergeCell ref="A4:B4"/>
     <mergeCell ref="E4:F4"/>
     <mergeCell ref="A5:B5"/>
     <mergeCell ref="E5:F5"/>
     <mergeCell ref="A6:B6"/>
     <mergeCell ref="E6:F6"/>
-    <mergeCell ref="A15:F15"/>
-    <mergeCell ref="A20:F20"/>
-    <mergeCell ref="A23:F23"/>
-    <mergeCell ref="A24:F24"/>
-    <mergeCell ref="A25:F25"/>
-    <mergeCell ref="A26:F26"/>
+    <mergeCell ref="A10:A13"/>
+    <mergeCell ref="B10:B13"/>
+    <mergeCell ref="H10:H13"/>
+    <mergeCell ref="A14:A17"/>
+    <mergeCell ref="B14:B17"/>
+    <mergeCell ref="H14:H17"/>
+    <mergeCell ref="A18:A21"/>
+    <mergeCell ref="B18:B21"/>
+    <mergeCell ref="H18:H21"/>
+    <mergeCell ref="A22:A25"/>
+    <mergeCell ref="B22:B25"/>
+    <mergeCell ref="H22:H25"/>
+    <mergeCell ref="A26:A29"/>
+    <mergeCell ref="B26:B29"/>
+    <mergeCell ref="H26:H29"/>
+    <mergeCell ref="A30:G30"/>
+    <mergeCell ref="A33:A36"/>
+    <mergeCell ref="B33:B36"/>
+    <mergeCell ref="H33:H36"/>
+    <mergeCell ref="A37:A40"/>
+    <mergeCell ref="B37:B40"/>
+    <mergeCell ref="H37:H40"/>
+    <mergeCell ref="A41:G41"/>
+    <mergeCell ref="A44:G44"/>
+    <mergeCell ref="A45:G45"/>
+    <mergeCell ref="A46:G46"/>
+    <mergeCell ref="A47:G47"/>
   </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="landscape" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter differentFirst="false" differentOddEven="false">
     <oddHeader/>
     <oddFooter/>

</xml_diff>

<commit_message>
Timesheet: add Hannah Plumbing and Heating logo
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01WkobnVQXdGo996siArThhM
</commit_message>
<xml_diff>
--- a/Weekly_Timesheet_Hannah_Plumbing.xlsx
+++ b/Weekly_Timesheet_Hannah_Plumbing.xlsx
@@ -71,10 +71,10 @@
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="89" uniqueCount="46">
   <si>
-    <t xml:space="preserve">HANNAH PLUMBING &amp; HEATING LTD - WEEKLY TIMESHEET</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Yellow cells are for the employee to fill in. Enter times as 24hr (e.g. 08:00, 16:30) and unpaid break in minutes. Hours are worked out automatically. Leave a day blank if not worked.</t>
+    <t xml:space="preserve">WEEKLY TIMESHEET</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Yellow cells are for the employee to fill in. Enter times as 24hr (e.g. 08:00, 16:30) and unpaid break in minutes. Hours are worked out automatically. Use one line per job (up to 4 a day); leave unused lines blank.</t>
   </si>
   <si>
     <t xml:space="preserve">Employee name</t>
@@ -247,7 +247,8 @@
     </font>
     <font>
       <b val="true"/>
-      <sz val="14"/>
+      <sz val="16"/>
+      <color rgb="FF0A0F7A"/>
       <name val="Arial"/>
       <family val="0"/>
       <charset val="1"/>
@@ -396,8 +397,8 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
@@ -521,7 +522,7 @@
       <rgbColor rgb="FF00FFFF"/>
       <rgbColor rgb="FF800000"/>
       <rgbColor rgb="FF008000"/>
-      <rgbColor rgb="FF000080"/>
+      <rgbColor rgb="FF0A0F7A"/>
       <rgbColor rgb="FF808000"/>
       <rgbColor rgb="FF800080"/>
       <rgbColor rgb="FF008080"/>
@@ -570,6 +571,90 @@
     </indexedColors>
   </colors>
 </styleSheet>
+</file>
+
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>2</xdr:col>
+      <xdr:colOff>142560</xdr:colOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>856800</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="0" name="Image 1" descr="Picture"/>
+        <xdr:cNvPicPr/>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip r:embed="rId1"/>
+        <a:stretch/>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="0" y="0"/>
+          <a:ext cx="1904760" cy="856800"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:ln w="0">
+          <a:noFill/>
+        </a:ln>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>2</xdr:col>
+      <xdr:colOff>142560</xdr:colOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>856800</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="1" name="Image 1" descr="Picture"/>
+        <xdr:cNvPicPr/>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip r:embed="rId1"/>
+        <a:stretch/>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="0" y="0"/>
+          <a:ext cx="1904760" cy="856800"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:ln w="0">
+          <a:noFill/>
+        </a:ln>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -764,12 +849,12 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="0" width="30"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="2" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="1" customFormat="false" ht="72" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="D1" s="1" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
         <v>1</v>
       </c>
@@ -1500,7 +1585,8 @@
     <oddHeader/>
     <oddFooter/>
   </headerFooter>
-  <legacyDrawing r:id="rId2"/>
+  <drawing r:id="rId2"/>
+  <legacyDrawing r:id="rId3"/>
 </worksheet>
 </file>
 
@@ -1521,12 +1607,12 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="0" width="30"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="2" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="1" customFormat="false" ht="72" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="D1" s="1" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
         <v>1</v>
       </c>
@@ -2327,6 +2413,7 @@
     <oddHeader/>
     <oddFooter/>
   </headerFooter>
-  <legacyDrawing r:id="rId2"/>
+  <drawing r:id="rId2"/>
+  <legacyDrawing r:id="rId3"/>
 </worksheet>
 </file>
</xml_diff>